<commit_message>
Re-skin Automation Playbook workbook: expense report coding example
</commit_message>
<xml_diff>
--- a/courser-university/automation/automation-playbook-workbook-template.xlsx
+++ b/courser-university/automation/automation-playbook-workbook-template.xlsx
@@ -568,7 +568,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2. Gray rows are the worked example — the 45-person firm's invoice-coding task. Overwrite nothing; type your own rows underneath.</t>
+          <t>2. Gray rows are the worked example — the 60-person firm's expense report coding task. Overwrite nothing; type your own rows underneath.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • Approach Pick            — Module 2 · CHOOSE: the task on the four-rung ladder</t>
+          <t xml:space="preserve">      • Approach Pick            — Module 2 · CHOOSE: the task on the four-level ladder</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Example — the firm's invoice-coding task</t>
+          <t>Example — the firm's expense report coding task</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       <c r="B5" s="12" t="n"/>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Code incoming vendor invoices to the right GL account</t>
+          <t>Code incoming employee expense reports to the right category</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="B6" s="12" t="n"/>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>The AP clerk, in Finance — about 6 hours a week</t>
+          <t>The bookkeeper, in Finance — about 6 hours a week</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       <c r="B7" s="12" t="n"/>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>The controller — signs the coding before it posts</t>
+          <t>The controller — signs the coding before it's reimbursed</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Payroll + vendor terms → money · Confidential</t>
+          <t>Payroll + merchant terms → money · Confidential</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Code vendor invoices to GL accounts</t>
+          <t>Code employee expense reports to expense categories</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Review the month-end close</t>
+          <t>Review which overdue accounts go to collections</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
@@ -1230,14 +1230,14 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>THE APPROACH PICK — place your task on the ladder; start on the lowest rung that does the job</t>
+          <t>THE APPROACH PICK — place your task on the ladder; start on the lowest level that does the job</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Four rungs, lightest first: 1 Prompt/agent recipe · 2 No-code workflow · 3 Connected integration · 4 Custom build. What pushes a task UP = integration surface + volume/durability, not enthusiasm.</t>
+          <t>Four levels, lightest first: 1 Prompt/agent recipe · 2 No-code workflow · 3 Connected integration · 4 Custom build. What pushes a task UP = integration surface + volume/durability, not enthusiasm.</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Rung (start lowest that works)</t>
+          <t>Level (start lowest that works)</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Why this rung</t>
+          <t>Why this level</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -1266,7 +1266,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Code vendor invoices to GL accounts</t>
+          <t>Code employee expense reports to expense categories</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Structured, repeatable, feeds one system; the SOP-Execution Agent drafts, the controller signs. A money-touch does NOT push it up — safety is the signature, not a heavier rung.</t>
+          <t>Structured, repeatable, feeds one system; the SOP-Execution Agent drafts, the controller signs. A money-touch does NOT push it up — safety is the signature, not a heavier level.</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Example — invoice coding</t>
+          <t>Example — expense report coding</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       <c r="B5" s="12" t="n"/>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Code incoming vendor invoices to the right GL account</t>
+          <t>Code incoming employee expense reports to the right category</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       <c r="B6" s="12" t="n"/>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>A new vendor invoice lands in the AP inbox</t>
+          <t>A new employee expense report lands in the AP inbox</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       <c r="B7" s="12" t="n"/>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>The invoice; the vendor→category list; the chart of accounts</t>
+          <t>The expense report; the the expense policy; the chart of accounts</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>1) Read vendor + line items. 2) Match vendor to its usual category. 3) Apply the GL rule for that category. 4) Produce a draft coding with the amount and account.</t>
+          <t>1) Read each expense line (merchant, amount, date). 2) Match it to a category. 3) Check it against the policy rule. 4) Produce a draft coding + a policy flag per line.</t>
         </is>
       </c>
     </row>
@@ -1465,20 +1465,20 @@
       <c r="B9" s="12" t="n"/>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Split invoice (2+ categories) → FLAG. New vendor not on the list → FLAG. A credit / credit memo → FLAG. Amount over threshold → FLAG for extra review.</t>
+          <t>Missing receipt (required over the policy threshold) → FLAG. Over-the-limit charge (above the per-diem / policy cap) → FLAG. A personal / non-reimbursable item → FLAG for the controller.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Sign-off (the named human, before anything posts)</t>
+          <t>Sign-off (the named human, before anything is reimbursed)</t>
         </is>
       </c>
       <c r="B10" s="12" t="n"/>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>The controller reviews the draft, edits if needed, and posts. The agent never posts, pays, or touches the ledger.</t>
+          <t>The controller reviews the draft, edits if needed, and approves the reimbursement. The agent never approves, pays, or issues a reimbursement.</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Example — invoice coding</t>
+          <t>Example — expense report coding</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
       <c r="B5" s="12" t="n"/>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>One vendor category only (software subscriptions) — not the whole AP inbox</t>
+          <t>One merchant category only (travel &amp;amp; meals) — not the whole AP inbox</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       <c r="B7" s="12" t="n"/>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Company accounts + approved AI only; drafts only — never touches the ledger or payment</t>
+          <t>Company accounts + approved AI only; drafts only — never approves or pays a reimbursement</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Confidential — payroll + vendor terms</t>
+          <t>Confidential — reimbursements + expense policy</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       <c r="B10" s="12" t="n"/>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Turn the agent off; the AP clerk codes manually — the way it always worked</t>
+          <t>Turn the agent off; the bookkeeper codes manually — the way it always worked</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Example — invoice coding (numbers are a labeled synthetic example)</t>
+          <t>Example — expense report coding (numbers are a labeled synthetic example)</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       <c r="B5" s="12" t="n"/>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Split invoice · new vendor · credit memo · over-threshold amount — plus a batch of ordinary ones</t>
+          <t>Missing receipt · over-the-limit charge · personal item · over-threshold amount — plus a batch of ordinary ones</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       <c r="B7" s="12" t="n"/>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>The AP clerk codes invoices by hand — no automation ships without this</t>
+          <t>The bookkeeper codes expense reports by hand — no automation ships without this</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>~6 hrs/week on the pilot category (measured over 2 weeks) — synthetic example</t>
+          <t>~5 hrs/week on the pilot category (measured over 2 weeks) — synthetic example</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
       <c r="B9" s="12" t="n"/>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>~2 hrs/week drafting + review — synthetic example</t>
+          <t>~1.5 hrs/week drafting + review — synthetic example</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       <c r="B10" s="12" t="n"/>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>~4 hrs/week back on this one category (estimate) — no 'average', no benchmark</t>
+          <t>~3.5 hrs/week back on this one category (estimate) — no 'average', no benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook snapshot: fix hours + touches residuals
</commit_message>
<xml_diff>
--- a/courser-university/automation/automation-playbook-workbook-template.xlsx
+++ b/courser-university/automation/automation-playbook-workbook-template.xlsx
@@ -741,7 +741,7 @@
       <c r="B6" s="12" t="n"/>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>The bookkeeper, in Finance — about 6 hours a week</t>
+          <t>The bookkeeper, in Finance — about 5 hours a week</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Payroll + merchant terms → money · Confidential</t>
+          <t>Reimbursements + expense policy → money · Confidential</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       <c r="B7" s="12" t="n"/>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>The expense report; the the expense policy; the chart of accounts</t>
+          <t>The expense report; the expense policy; the chart of accounts</t>
         </is>
       </c>
     </row>

</xml_diff>